<commit_message>
Adjust type in /History/TimeSinceLastFullCharge
It is an uint32 instead of an uint16.
</commit_message>
<xml_diff>
--- a/CCGX-Modbus-TCP-register-list.xlsx
+++ b/CCGX-Modbus-TCP-register-list.xlsx
@@ -5,12 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Field list" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Unit ID mapping" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Document versions" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Field list" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Unit ID mapping" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Document versions" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -4976,7 +4976,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5066,10 +5066,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5178,17 +5174,123 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N1048576"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="37.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="8.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="26.6"/>
@@ -10432,7 +10534,7 @@
         <v>289</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>20</v>
+        <v>341</v>
       </c>
       <c r="E173" s="1" t="n">
         <v>0.01</v>
@@ -16609,7 +16711,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="382" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A382" s="1" t="s">
         <v>835</v>
       </c>
@@ -16735,7 +16837,7 @@
       <c r="A386" s="1" t="s">
         <v>806</v>
       </c>
-      <c r="B386" s="23" t="s">
+      <c r="B386" s="22" t="s">
         <v>849</v>
       </c>
       <c r="C386" s="1" t="n">
@@ -16744,7 +16846,7 @@
       <c r="D386" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E386" s="23" t="n">
+      <c r="E386" s="22" t="n">
         <v>1</v>
       </c>
       <c r="F386" s="3" t="s">
@@ -16764,7 +16866,7 @@
       <c r="A387" s="1" t="s">
         <v>806</v>
       </c>
-      <c r="B387" s="23" t="s">
+      <c r="B387" s="22" t="s">
         <v>852</v>
       </c>
       <c r="C387" s="1" t="n">
@@ -16773,7 +16875,7 @@
       <c r="D387" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E387" s="23" t="n">
+      <c r="E387" s="22" t="n">
         <v>1</v>
       </c>
       <c r="F387" s="3" t="s">
@@ -16793,7 +16895,7 @@
       <c r="A388" s="1" t="s">
         <v>806</v>
       </c>
-      <c r="B388" s="23" t="s">
+      <c r="B388" s="22" t="s">
         <v>854</v>
       </c>
       <c r="C388" s="1" t="n">
@@ -16802,7 +16904,7 @@
       <c r="D388" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E388" s="23" t="n">
+      <c r="E388" s="22" t="n">
         <v>1</v>
       </c>
       <c r="F388" s="3" t="s">
@@ -16818,7 +16920,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="389" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="1" t="s">
         <v>835</v>
       </c>
@@ -16831,7 +16933,7 @@
       <c r="D389" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="E389" s="23" t="n">
+      <c r="E389" s="22" t="n">
         <v>1</v>
       </c>
       <c r="F389" s="3" t="s">
@@ -17198,7 +17300,7 @@
       <c r="H401" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I401" s="24"/>
+      <c r="I401" s="23"/>
     </row>
     <row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="1" t="s">
@@ -27749,19 +27851,19 @@
       <c r="B773" s="1" t="s">
         <v>1229</v>
       </c>
-      <c r="C773" s="25" t="n">
+      <c r="C773" s="24" t="n">
         <v>5200</v>
       </c>
-      <c r="D773" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E773" s="25" t="n">
+      <c r="D773" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E773" s="24" t="n">
         <v>1</v>
       </c>
       <c r="F773" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="G773" s="25" t="s">
+      <c r="G773" s="24" t="s">
         <v>898</v>
       </c>
       <c r="H773" s="1" t="s">
@@ -27775,19 +27877,19 @@
       <c r="B774" s="1" t="s">
         <v>973</v>
       </c>
-      <c r="C774" s="25" t="n">
+      <c r="C774" s="24" t="n">
         <v>5201</v>
       </c>
-      <c r="D774" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E774" s="25" t="n">
+      <c r="D774" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E774" s="24" t="n">
         <v>1</v>
       </c>
       <c r="F774" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="G774" s="25" t="s">
+      <c r="G774" s="24" t="s">
         <v>974</v>
       </c>
       <c r="H774" s="1" t="s">
@@ -27801,19 +27903,19 @@
       <c r="B775" s="1" t="s">
         <v>676</v>
       </c>
-      <c r="C775" s="25" t="n">
+      <c r="C775" s="24" t="n">
         <v>5202</v>
       </c>
-      <c r="D775" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E775" s="25" t="n">
+      <c r="D775" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E775" s="24" t="n">
         <v>1</v>
       </c>
       <c r="F775" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="G775" s="25" t="s">
+      <c r="G775" s="24" t="s">
         <v>564</v>
       </c>
       <c r="H775" s="1" t="s">
@@ -27827,19 +27929,19 @@
       <c r="B776" s="1" t="s">
         <v>1211</v>
       </c>
-      <c r="C776" s="25" t="n">
+      <c r="C776" s="24" t="n">
         <v>5203</v>
       </c>
-      <c r="D776" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E776" s="25" t="n">
+      <c r="D776" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E776" s="24" t="n">
         <v>1</v>
       </c>
       <c r="F776" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="G776" s="25" t="s">
+      <c r="G776" s="24" t="s">
         <v>978</v>
       </c>
       <c r="H776" s="1" t="s">
@@ -27853,19 +27955,19 @@
       <c r="B777" s="1" t="s">
         <v>993</v>
       </c>
-      <c r="C777" s="25" t="n">
+      <c r="C777" s="24" t="n">
         <v>5204</v>
       </c>
-      <c r="D777" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E777" s="25" t="n">
+      <c r="D777" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E777" s="24" t="n">
         <v>1</v>
       </c>
       <c r="F777" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="G777" s="25" t="s">
+      <c r="G777" s="24" t="s">
         <v>994</v>
       </c>
       <c r="H777" s="1" t="s">
@@ -27882,19 +27984,19 @@
       <c r="B778" s="1" t="s">
         <v>1230</v>
       </c>
-      <c r="C778" s="25" t="n">
+      <c r="C778" s="24" t="n">
         <v>5205</v>
       </c>
-      <c r="D778" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E778" s="25" t="n">
+      <c r="D778" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E778" s="24" t="n">
         <v>100</v>
       </c>
       <c r="F778" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="G778" s="25" t="s">
+      <c r="G778" s="24" t="s">
         <v>213</v>
       </c>
       <c r="H778" s="1" t="s">
@@ -27911,19 +28013,19 @@
       <c r="B779" s="1" t="s">
         <v>1232</v>
       </c>
-      <c r="C779" s="25" t="n">
+      <c r="C779" s="24" t="n">
         <v>5206</v>
       </c>
-      <c r="D779" s="25" t="s">
+      <c r="D779" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E779" s="25" t="n">
+      <c r="E779" s="24" t="n">
         <v>10</v>
       </c>
       <c r="F779" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G779" s="25" t="s">
+      <c r="G779" s="24" t="s">
         <v>215</v>
       </c>
       <c r="H779" s="1" t="s">
@@ -27937,22 +28039,22 @@
       <c r="A780" s="22" t="s">
         <v>1228</v>
       </c>
-      <c r="B780" s="25" t="s">
+      <c r="B780" s="24" t="s">
         <v>979</v>
       </c>
-      <c r="C780" s="25" t="n">
+      <c r="C780" s="24" t="n">
         <v>5207</v>
       </c>
-      <c r="D780" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E780" s="25" t="n">
+      <c r="D780" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E780" s="24" t="n">
         <v>1</v>
       </c>
       <c r="F780" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="G780" s="25" t="s">
+      <c r="G780" s="24" t="s">
         <v>980</v>
       </c>
       <c r="H780" s="1" t="s">
@@ -27969,19 +28071,19 @@
       <c r="B781" s="1" t="s">
         <v>1234</v>
       </c>
-      <c r="C781" s="25" t="n">
+      <c r="C781" s="24" t="n">
         <v>5208</v>
       </c>
-      <c r="D781" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E781" s="25" t="n">
+      <c r="D781" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E781" s="24" t="n">
         <v>1</v>
       </c>
       <c r="F781" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="G781" s="25" t="s">
+      <c r="G781" s="24" t="s">
         <v>982</v>
       </c>
       <c r="H781" s="1" t="s">
@@ -27998,19 +28100,19 @@
       <c r="B782" s="1" t="s">
         <v>1000</v>
       </c>
-      <c r="C782" s="25" t="n">
+      <c r="C782" s="24" t="n">
         <v>5209</v>
       </c>
-      <c r="D782" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E782" s="25" t="s">
+      <c r="D782" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E782" s="24" t="s">
         <v>1235</v>
       </c>
       <c r="F782" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="G782" s="25" t="s">
+      <c r="G782" s="24" t="s">
         <v>984</v>
       </c>
       <c r="H782" s="1" t="s">
@@ -28024,22 +28126,22 @@
       <c r="A783" s="22" t="s">
         <v>1228</v>
       </c>
-      <c r="B783" s="25" t="s">
+      <c r="B783" s="24" t="s">
         <v>985</v>
       </c>
-      <c r="C783" s="25" t="n">
+      <c r="C783" s="24" t="n">
         <v>5210</v>
       </c>
-      <c r="D783" s="25" t="s">
+      <c r="D783" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E783" s="25" t="n">
+      <c r="E783" s="24" t="n">
         <v>10</v>
       </c>
       <c r="F783" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G783" s="25" t="s">
+      <c r="G783" s="24" t="s">
         <v>986</v>
       </c>
       <c r="H783" s="1" t="s">
@@ -28053,22 +28155,22 @@
       <c r="A784" s="22" t="s">
         <v>1228</v>
       </c>
-      <c r="B784" s="25" t="s">
+      <c r="B784" s="24" t="s">
         <v>1237</v>
       </c>
-      <c r="C784" s="25" t="n">
+      <c r="C784" s="24" t="n">
         <v>5211</v>
       </c>
-      <c r="D784" s="25" t="s">
+      <c r="D784" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E784" s="25" t="n">
+      <c r="E784" s="24" t="n">
         <v>10</v>
       </c>
       <c r="F784" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G784" s="25" t="s">
+      <c r="G784" s="24" t="s">
         <v>988</v>
       </c>
       <c r="H784" s="1" t="s">
@@ -28082,22 +28184,22 @@
       <c r="A785" s="22" t="s">
         <v>1228</v>
       </c>
-      <c r="B785" s="25" t="s">
+      <c r="B785" s="24" t="s">
         <v>989</v>
       </c>
-      <c r="C785" s="25" t="n">
+      <c r="C785" s="24" t="n">
         <v>5212</v>
       </c>
-      <c r="D785" s="25" t="s">
+      <c r="D785" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E785" s="25" t="n">
+      <c r="E785" s="24" t="n">
         <v>10</v>
       </c>
       <c r="F785" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G785" s="25" t="s">
+      <c r="G785" s="24" t="s">
         <v>990</v>
       </c>
       <c r="H785" s="1" t="s">
@@ -28111,22 +28213,22 @@
       <c r="A786" s="22" t="s">
         <v>1228</v>
       </c>
-      <c r="B786" s="25" t="s">
+      <c r="B786" s="24" t="s">
         <v>400</v>
       </c>
-      <c r="C786" s="25" t="n">
+      <c r="C786" s="24" t="n">
         <v>5213</v>
       </c>
-      <c r="D786" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E786" s="25" t="n">
+      <c r="D786" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E786" s="24" t="n">
         <v>100</v>
       </c>
       <c r="F786" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="G786" s="25" t="s">
+      <c r="G786" s="24" t="s">
         <v>992</v>
       </c>
       <c r="H786" s="1" t="s">
@@ -28143,19 +28245,19 @@
       <c r="B787" s="1" t="s">
         <v>997</v>
       </c>
-      <c r="C787" s="25" t="n">
+      <c r="C787" s="24" t="n">
         <v>5214</v>
       </c>
-      <c r="D787" s="25" t="s">
+      <c r="D787" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E787" s="25" t="n">
+      <c r="E787" s="24" t="n">
         <v>1</v>
       </c>
       <c r="F787" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G787" s="25" t="s">
+      <c r="G787" s="24" t="s">
         <v>998</v>
       </c>
       <c r="H787" s="1" t="s">
@@ -28169,22 +28271,22 @@
       <c r="A788" s="22" t="s">
         <v>1228</v>
       </c>
-      <c r="B788" s="25" t="s">
+      <c r="B788" s="24" t="s">
         <v>1234</v>
       </c>
-      <c r="C788" s="25" t="n">
+      <c r="C788" s="24" t="n">
         <v>5215</v>
       </c>
-      <c r="D788" s="25" t="s">
+      <c r="D788" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E788" s="25" t="n">
+      <c r="E788" s="24" t="n">
         <v>10</v>
       </c>
       <c r="F788" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G788" s="25" t="s">
+      <c r="G788" s="24" t="s">
         <v>1238</v>
       </c>
       <c r="H788" s="1" t="s">
@@ -28201,19 +28303,19 @@
       <c r="B789" s="1" t="s">
         <v>1000</v>
       </c>
-      <c r="C789" s="25" t="n">
+      <c r="C789" s="24" t="n">
         <v>5216</v>
       </c>
-      <c r="D789" s="25" t="s">
+      <c r="D789" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E789" s="25" t="n">
+      <c r="E789" s="24" t="n">
         <v>1</v>
       </c>
       <c r="F789" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G789" s="25" t="s">
+      <c r="G789" s="24" t="s">
         <v>1001</v>
       </c>
       <c r="H789" s="1" t="s">
@@ -28227,19 +28329,19 @@
       <c r="A790" s="22" t="s">
         <v>1228</v>
       </c>
-      <c r="B790" s="25" t="s">
+      <c r="B790" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="C790" s="25" t="n">
+      <c r="C790" s="24" t="n">
         <v>5217</v>
       </c>
-      <c r="D790" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E790" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G790" s="25" t="s">
+      <c r="D790" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E790" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G790" s="24" t="s">
         <v>130</v>
       </c>
       <c r="H790" s="1" t="s">
@@ -28253,16 +28355,16 @@
       <c r="B791" s="1" t="s">
         <v>1002</v>
       </c>
-      <c r="C791" s="25" t="n">
+      <c r="C791" s="24" t="n">
         <v>5218</v>
       </c>
-      <c r="D791" s="25" t="s">
+      <c r="D791" s="24" t="s">
         <v>1003</v>
       </c>
-      <c r="E791" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G791" s="25" t="s">
+      <c r="E791" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G791" s="24" t="s">
         <v>1005</v>
       </c>
       <c r="H791" s="1" t="s">
@@ -28279,16 +28381,16 @@
       <c r="B792" s="1" t="s">
         <v>1007</v>
       </c>
-      <c r="C792" s="25" t="n">
+      <c r="C792" s="24" t="n">
         <v>5234</v>
       </c>
-      <c r="D792" s="25" t="s">
+      <c r="D792" s="24" t="s">
         <v>1003</v>
       </c>
-      <c r="E792" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G792" s="25" t="s">
+      <c r="E792" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G792" s="24" t="s">
         <v>1008</v>
       </c>
       <c r="H792" s="1" t="s">
@@ -28302,16 +28404,16 @@
       <c r="B793" s="1" t="s">
         <v>1009</v>
       </c>
-      <c r="C793" s="25" t="n">
+      <c r="C793" s="24" t="n">
         <v>5250</v>
       </c>
-      <c r="D793" s="25" t="s">
+      <c r="D793" s="24" t="s">
         <v>1003</v>
       </c>
-      <c r="E793" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G793" s="25" t="s">
+      <c r="E793" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G793" s="24" t="s">
         <v>1010</v>
       </c>
       <c r="H793" s="1" t="s">
@@ -28325,16 +28427,16 @@
       <c r="B794" s="1" t="s">
         <v>1011</v>
       </c>
-      <c r="C794" s="25" t="n">
+      <c r="C794" s="24" t="n">
         <v>5266</v>
       </c>
-      <c r="D794" s="25" t="s">
+      <c r="D794" s="24" t="s">
         <v>1003</v>
       </c>
-      <c r="E794" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G794" s="25" t="s">
+      <c r="E794" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G794" s="24" t="s">
         <v>1012</v>
       </c>
       <c r="H794" s="1" t="s">
@@ -28348,16 +28450,16 @@
       <c r="B795" s="1" t="s">
         <v>1013</v>
       </c>
-      <c r="C795" s="25" t="n">
+      <c r="C795" s="24" t="n">
         <v>5282</v>
       </c>
-      <c r="D795" s="25" t="s">
+      <c r="D795" s="24" t="s">
         <v>1003</v>
       </c>
-      <c r="E795" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G795" s="25" t="s">
+      <c r="E795" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G795" s="24" t="s">
         <v>1014</v>
       </c>
       <c r="H795" s="1" t="s">
@@ -28371,16 +28473,16 @@
       <c r="B796" s="1" t="s">
         <v>1015</v>
       </c>
-      <c r="C796" s="25" t="n">
+      <c r="C796" s="24" t="n">
         <v>5298</v>
       </c>
-      <c r="D796" s="25" t="s">
+      <c r="D796" s="24" t="s">
         <v>1003</v>
       </c>
-      <c r="E796" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G796" s="25" t="s">
+      <c r="E796" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G796" s="24" t="s">
         <v>1016</v>
       </c>
       <c r="H796" s="1" t="s">
@@ -28394,16 +28496,16 @@
       <c r="B797" s="1" t="s">
         <v>1017</v>
       </c>
-      <c r="C797" s="25" t="n">
+      <c r="C797" s="24" t="n">
         <v>5314</v>
       </c>
-      <c r="D797" s="25" t="s">
+      <c r="D797" s="24" t="s">
         <v>1003</v>
       </c>
-      <c r="E797" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G797" s="25" t="s">
+      <c r="E797" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G797" s="24" t="s">
         <v>1018</v>
       </c>
       <c r="H797" s="1" t="s">
@@ -28417,16 +28519,16 @@
       <c r="B798" s="1" t="s">
         <v>1019</v>
       </c>
-      <c r="C798" s="25" t="n">
+      <c r="C798" s="24" t="n">
         <v>5330</v>
       </c>
-      <c r="D798" s="25" t="s">
+      <c r="D798" s="24" t="s">
         <v>1003</v>
       </c>
-      <c r="E798" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G798" s="25" t="s">
+      <c r="E798" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G798" s="24" t="s">
         <v>1020</v>
       </c>
       <c r="H798" s="1" t="s">
@@ -28437,7 +28539,7 @@
       <c r="A799" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B799" s="25" t="s">
+      <c r="B799" s="24" t="s">
         <v>1239</v>
       </c>
       <c r="C799" s="1" t="n">
@@ -28524,7 +28626,7 @@
       <c r="A802" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B802" s="26" t="s">
+      <c r="B802" s="25" t="s">
         <v>1248</v>
       </c>
       <c r="C802" s="1" t="n">
@@ -28968,8 +29070,8 @@
     <hyperlink ref="I791" r:id="rId3" location="error-codes" display="See https://github.com/victronenergy/venus/wiki/dbus#error-codes"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -28978,27 +29080,27 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F1048576"/>
-  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="22" width="7.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="22" width="7.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="22" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="22" width="65.01"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="4" style="22" width="8.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>1284</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="26" t="s">
         <v>1285</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="26" t="s">
         <v>1286</v>
       </c>
     </row>
@@ -29166,24 +29268,24 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28" t="n">
+      <c r="A22" s="27" t="n">
         <v>223</v>
       </c>
-      <c r="B22" s="28" t="n">
+      <c r="B22" s="27" t="n">
         <v>277</v>
       </c>
-      <c r="C22" s="28" t="s">
+      <c r="C22" s="27" t="s">
         <v>1288</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28" t="n">
+      <c r="A23" s="27" t="n">
         <v>224</v>
       </c>
-      <c r="B23" s="28" t="n">
+      <c r="B23" s="27" t="n">
         <v>278</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="27" t="s">
         <v>1289</v>
       </c>
     </row>
@@ -29199,57 +29301,57 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="28" t="n">
+      <c r="A25" s="27" t="n">
         <v>226</v>
       </c>
-      <c r="B25" s="28" t="n">
+      <c r="B25" s="27" t="n">
         <v>279</v>
       </c>
-      <c r="C25" s="28" t="s">
+      <c r="C25" s="27" t="s">
         <v>1291</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="28" t="n">
+      <c r="A26" s="27" t="n">
         <v>227</v>
       </c>
-      <c r="B26" s="28" t="n">
+      <c r="B26" s="27" t="n">
         <v>276</v>
       </c>
-      <c r="C26" s="28" t="s">
+      <c r="C26" s="27" t="s">
         <v>1292</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="28" t="n">
+      <c r="A27" s="27" t="n">
         <v>228</v>
       </c>
-      <c r="B27" s="28" t="n">
+      <c r="B27" s="27" t="n">
         <v>275</v>
       </c>
-      <c r="C27" s="28" t="s">
+      <c r="C27" s="27" t="s">
         <v>1293</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="28" t="n">
+      <c r="A28" s="27" t="n">
         <v>229</v>
       </c>
-      <c r="B28" s="28" t="n">
+      <c r="B28" s="27" t="n">
         <v>274</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="27" t="s">
         <v>1294</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="28" t="n">
+      <c r="A29" s="27" t="n">
         <v>230</v>
       </c>
-      <c r="B29" s="28" t="n">
+      <c r="B29" s="27" t="n">
         <v>273</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="27" t="s">
         <v>1295</v>
       </c>
     </row>
@@ -29353,35 +29455,35 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="28" t="n">
+      <c r="A39" s="27" t="n">
         <v>242</v>
       </c>
-      <c r="B39" s="28" t="n">
+      <c r="B39" s="27" t="n">
         <v>261</v>
       </c>
-      <c r="C39" s="28" t="s">
+      <c r="C39" s="27" t="s">
         <v>1305</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="28" t="n">
+      <c r="A40" s="27" t="n">
         <v>243</v>
       </c>
-      <c r="B40" s="28" t="n">
+      <c r="B40" s="27" t="n">
         <v>260</v>
       </c>
-      <c r="C40" s="28" t="s">
+      <c r="C40" s="27" t="s">
         <v>1306</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="28" t="n">
+      <c r="A41" s="27" t="n">
         <v>244</v>
       </c>
-      <c r="B41" s="28" t="n">
-        <v>259</v>
-      </c>
-      <c r="C41" s="28"/>
+      <c r="B41" s="27" t="n">
+        <v>259</v>
+      </c>
+      <c r="C41" s="27"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22" t="n">
@@ -29390,7 +29492,7 @@
       <c r="B42" s="22" t="n">
         <v>258</v>
       </c>
-      <c r="C42" s="28" t="s">
+      <c r="C42" s="27" t="s">
         <v>1307</v>
       </c>
     </row>
@@ -29417,24 +29519,24 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="29" t="s">
+      <c r="A46" s="28" t="s">
         <v>1310</v>
       </c>
-      <c r="B46" s="29"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="29"/>
-      <c r="E46" s="29"/>
-      <c r="F46" s="29"/>
+      <c r="B46" s="28"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="28"/>
+      <c r="F46" s="28"/>
     </row>
     <row r="47" customFormat="false" ht="92.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="30" t="s">
+      <c r="A47" s="29" t="s">
         <v>1311</v>
       </c>
-      <c r="B47" s="30"/>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="E47" s="30"/>
-      <c r="F47" s="30"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="29"/>
+      <c r="F47" s="29"/>
     </row>
     <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -29456,8 +29558,8 @@
     <mergeCell ref="A47:F47"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -29466,12 +29568,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C1048576"/>
-  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="22" width="8.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="22" width="3.43"/>
@@ -29703,7 +29805,7 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="54.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C39" s="31" t="s">
+      <c r="C39" s="30" t="s">
         <v>1361</v>
       </c>
     </row>
@@ -30407,8 +30509,8 @@
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
Fix swapped labels in DESS restrictions
Reported via https://community.victronenergy.com/t/node-red-restrictions-nodes-documentation-bug/53688
</commit_message>
<xml_diff>
--- a/CCGX-Modbus-TCP-register-list.xlsx
+++ b/CCGX-Modbus-TCP-register-list.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6798" uniqueCount="1691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6798" uniqueCount="1692">
   <si>
     <t xml:space="preserve">NOTE: Use unit-id 100 for the com.victronenergy.system data, for more information see FAQ.</t>
   </si>
@@ -4531,6 +4531,9 @@
   </si>
   <si>
     <t xml:space="preserve">/Settings/DynamicEss/Schedule/0/Restrictions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0=No restrictions between battery and the grid;1=Battery to grid energy flow is restricted;2=Grid to battery energy flow is restricted;3=No energy flow between battery and grid</t>
   </si>
   <si>
     <t xml:space="preserve">Target SOC for this schedule</t>
@@ -5866,7 +5869,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N960"/>
-  <sheetFormatPr defaultColWidth="9.01171875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.01171875" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="37.43"/>
@@ -5893,7 +5896,7 @@
       <c r="G1" s="8"/>
       <c r="H1" s="9"/>
     </row>
-    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
         <v>2</v>
       </c>
@@ -20038,7 +20041,7 @@
       </c>
       <c r="J479" s="21"/>
     </row>
-    <row r="480" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="480" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A480" s="21" t="s">
         <v>912</v>
       </c>
@@ -22844,7 +22847,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="579" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="579" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A579" s="1" t="s">
         <v>1069</v>
       </c>
@@ -22870,7 +22873,7 @@
         <v>1117</v>
       </c>
     </row>
-    <row r="580" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="580" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A580" s="1" t="s">
         <v>1069</v>
       </c>
@@ -22893,7 +22896,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="581" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="581" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A581" s="1" t="s">
         <v>1069</v>
       </c>
@@ -22916,7 +22919,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="582" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="582" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A582" s="1" t="s">
         <v>1069</v>
       </c>
@@ -22939,7 +22942,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="583" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="583" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A583" s="1" t="s">
         <v>1069</v>
       </c>
@@ -22962,7 +22965,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="584" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="584" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A584" s="1" t="s">
         <v>1069</v>
       </c>
@@ -22985,7 +22988,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="585" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="585" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A585" s="1" t="s">
         <v>1069</v>
       </c>
@@ -23008,7 +23011,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="586" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="586" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A586" s="1" t="s">
         <v>1069</v>
       </c>
@@ -23292,7 +23295,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="596" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="596" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A596" s="1" t="s">
         <v>1132</v>
       </c>
@@ -23324,7 +23327,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="597" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="597" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A597" s="1" t="s">
         <v>1132</v>
       </c>
@@ -23356,7 +23359,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="598" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="598" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A598" s="1" t="s">
         <v>1132</v>
       </c>
@@ -23385,7 +23388,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="599" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="599" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A599" s="1" t="s">
         <v>1132</v>
       </c>
@@ -23417,7 +23420,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="600" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="600" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A600" s="1" t="s">
         <v>1132</v>
       </c>
@@ -32316,7 +32319,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="921" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="921" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A921" s="22" t="s">
         <v>1363</v>
       </c>
@@ -32342,7 +32345,7 @@
         <v>1117</v>
       </c>
     </row>
-    <row r="922" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="922" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A922" s="22" t="s">
         <v>1363</v>
       </c>
@@ -32365,7 +32368,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="923" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="923" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A923" s="22" t="s">
         <v>1363</v>
       </c>
@@ -32388,7 +32391,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="924" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="924" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A924" s="22" t="s">
         <v>1363</v>
       </c>
@@ -32411,7 +32414,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="925" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="925" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A925" s="22" t="s">
         <v>1363</v>
       </c>
@@ -32434,7 +32437,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="926" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="926" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A926" s="22" t="s">
         <v>1363</v>
       </c>
@@ -32457,7 +32460,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="927" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="927" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A927" s="22" t="s">
         <v>1363</v>
       </c>
@@ -32480,7 +32483,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="928" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="928" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A928" s="22" t="s">
         <v>1363</v>
       </c>
@@ -32590,7 +32593,7 @@
         <v>1382</v>
       </c>
     </row>
-    <row r="932" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="932" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A932" s="1" t="s">
         <v>12</v>
       </c>
@@ -32932,7 +32935,7 @@
         <v>23</v>
       </c>
       <c r="I943" s="1" t="s">
-        <v>1390</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="944" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32940,7 +32943,7 @@
         <v>912</v>
       </c>
       <c r="B944" s="1" t="s">
-        <v>1413</v>
+        <v>1414</v>
       </c>
       <c r="C944" s="1" t="n">
         <v>5427</v>
@@ -32955,7 +32958,7 @@
         <v>264</v>
       </c>
       <c r="G944" s="1" t="s">
-        <v>1414</v>
+        <v>1415</v>
       </c>
       <c r="H944" s="1" t="s">
         <v>23</v>
@@ -32969,7 +32972,7 @@
         <v>912</v>
       </c>
       <c r="B945" s="1" t="s">
-        <v>1415</v>
+        <v>1416</v>
       </c>
       <c r="C945" s="1" t="n">
         <v>5428</v>
@@ -32984,7 +32987,7 @@
         <v>140</v>
       </c>
       <c r="G945" s="1" t="s">
-        <v>1416</v>
+        <v>1417</v>
       </c>
       <c r="H945" s="1" t="s">
         <v>23</v>
@@ -32995,7 +32998,7 @@
         <v>912</v>
       </c>
       <c r="B946" s="1" t="s">
-        <v>1417</v>
+        <v>1418</v>
       </c>
       <c r="C946" s="1" t="n">
         <v>5429</v>
@@ -33010,7 +33013,7 @@
         <v>264</v>
       </c>
       <c r="G946" s="1" t="s">
-        <v>1418</v>
+        <v>1419</v>
       </c>
       <c r="H946" s="1" t="s">
         <v>23</v>
@@ -33021,7 +33024,7 @@
     </row>
     <row r="947" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A947" s="1" t="s">
-        <v>1419</v>
+        <v>1420</v>
       </c>
       <c r="B947" s="1" t="s">
         <v>1006</v>
@@ -33047,10 +33050,10 @@
     </row>
     <row r="948" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A948" s="1" t="s">
-        <v>1419</v>
+        <v>1420</v>
       </c>
       <c r="B948" s="1" t="s">
-        <v>1420</v>
+        <v>1421</v>
       </c>
       <c r="C948" s="1" t="n">
         <v>5501</v>
@@ -33071,15 +33074,15 @@
         <v>17</v>
       </c>
       <c r="I948" s="1" t="s">
-        <v>1421</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="949" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A949" s="1" t="s">
-        <v>1419</v>
+        <v>1420</v>
       </c>
       <c r="B949" s="1" t="s">
-        <v>1422</v>
+        <v>1423</v>
       </c>
       <c r="C949" s="1" t="n">
         <v>5502</v>
@@ -33105,7 +33108,7 @@
     </row>
     <row r="950" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A950" s="1" t="s">
-        <v>1419</v>
+        <v>1420</v>
       </c>
       <c r="B950" s="1" t="s">
         <v>1271</v>
@@ -33134,10 +33137,10 @@
     </row>
     <row r="951" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A951" s="1" t="s">
-        <v>1419</v>
+        <v>1420</v>
       </c>
       <c r="B951" s="1" t="s">
-        <v>1423</v>
+        <v>1424</v>
       </c>
       <c r="C951" s="1" t="n">
         <v>5506</v>
@@ -33163,10 +33166,10 @@
     </row>
     <row r="952" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A952" s="1" t="s">
-        <v>1419</v>
+        <v>1420</v>
       </c>
       <c r="B952" s="1" t="s">
-        <v>1424</v>
+        <v>1425</v>
       </c>
       <c r="C952" s="1" t="n">
         <v>5507</v>
@@ -33181,7 +33184,7 @@
         <v>94</v>
       </c>
       <c r="G952" s="1" t="s">
-        <v>1425</v>
+        <v>1426</v>
       </c>
       <c r="H952" s="1" t="s">
         <v>17</v>
@@ -33192,10 +33195,10 @@
     </row>
     <row r="953" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A953" s="1" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="B953" s="27" t="s">
-        <v>1427</v>
+        <v>1428</v>
       </c>
       <c r="C953" s="1" t="n">
         <v>5800</v>
@@ -33210,21 +33213,21 @@
         <v>264</v>
       </c>
       <c r="G953" s="1" t="s">
-        <v>1428</v>
+        <v>1429</v>
       </c>
       <c r="H953" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I953" s="1" t="s">
-        <v>1429</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="954" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A954" s="1" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="B954" s="1" t="s">
-        <v>1430</v>
+        <v>1431</v>
       </c>
       <c r="C954" s="1" t="n">
         <v>5801</v>
@@ -33239,21 +33242,21 @@
         <v>264</v>
       </c>
       <c r="G954" s="1" t="s">
-        <v>1431</v>
+        <v>1432</v>
       </c>
       <c r="H954" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I954" s="1" t="s">
-        <v>1432</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="955" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A955" s="1" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="B955" s="1" t="s">
-        <v>1433</v>
+        <v>1434</v>
       </c>
       <c r="C955" s="1" t="n">
         <v>5802</v>
@@ -33268,32 +33271,32 @@
         <v>264</v>
       </c>
       <c r="G955" s="1" t="s">
-        <v>1434</v>
+        <v>1435</v>
       </c>
       <c r="H955" s="1" t="s">
         <v>17</v>
       </c>
       <c r="I955" s="1" t="s">
-        <v>1435</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="956" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A956" s="1" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="B956" s="27" t="s">
         <v>134</v>
       </c>
       <c r="C956" s="28" t="s">
-        <v>1436</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="957" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A957" s="1" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="B957" s="27" t="s">
-        <v>1427</v>
+        <v>1428</v>
       </c>
       <c r="C957" s="1" t="n">
         <v>5810</v>
@@ -33308,21 +33311,21 @@
         <v>264</v>
       </c>
       <c r="G957" s="1" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
       <c r="H957" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I957" s="1" t="s">
-        <v>1429</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="958" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A958" s="1" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="B958" s="1" t="s">
-        <v>1430</v>
+        <v>1431</v>
       </c>
       <c r="C958" s="1" t="n">
         <v>5811</v>
@@ -33337,21 +33340,21 @@
         <v>264</v>
       </c>
       <c r="G958" s="1" t="s">
-        <v>1438</v>
+        <v>1439</v>
       </c>
       <c r="H958" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I958" s="1" t="s">
-        <v>1432</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="959" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A959" s="1" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="B959" s="1" t="s">
-        <v>1433</v>
+        <v>1434</v>
       </c>
       <c r="C959" s="1" t="n">
         <v>5812</v>
@@ -33366,24 +33369,24 @@
         <v>264</v>
       </c>
       <c r="G959" s="1" t="s">
-        <v>1439</v>
+        <v>1440</v>
       </c>
       <c r="H959" s="1" t="s">
         <v>17</v>
       </c>
       <c r="I959" s="1" t="s">
-        <v>1435</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="960" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A960" s="1" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="B960" s="27" t="s">
         <v>134</v>
       </c>
       <c r="C960" s="28" t="s">
-        <v>1440</v>
+        <v>1441</v>
       </c>
     </row>
   </sheetData>
@@ -33411,7 +33414,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F1048576"/>
-  <sheetFormatPr defaultColWidth="8.578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.578125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="22" width="8.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="22" width="16"/>
@@ -33421,7 +33424,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="29" t="s">
-        <v>1441</v>
+        <v>1442</v>
       </c>
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
@@ -33431,7 +33434,7 @@
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="30" t="s">
-        <v>1442</v>
+        <v>1443</v>
       </c>
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
@@ -33446,7 +33449,7 @@
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="30" t="s">
-        <v>1443</v>
+        <v>1444</v>
       </c>
       <c r="B4" s="30"/>
       <c r="C4" s="30"/>
@@ -33466,13 +33469,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="31" t="s">
-        <v>1444</v>
+        <v>1445</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33483,7 +33486,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33646,7 +33649,7 @@
         <v>277</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33657,7 +33660,7 @@
         <v>278</v>
       </c>
       <c r="C29" s="30" t="s">
-        <v>1449</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33668,7 +33671,7 @@
         <v>512</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>1450</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33679,7 +33682,7 @@
         <v>279</v>
       </c>
       <c r="C31" s="30" t="s">
-        <v>1451</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33690,7 +33693,7 @@
         <v>276</v>
       </c>
       <c r="C32" s="30" t="s">
-        <v>1452</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33701,7 +33704,7 @@
         <v>275</v>
       </c>
       <c r="C33" s="30" t="s">
-        <v>1453</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33712,7 +33715,7 @@
         <v>274</v>
       </c>
       <c r="C34" s="30" t="s">
-        <v>1454</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33723,7 +33726,7 @@
         <v>273</v>
       </c>
       <c r="C35" s="30" t="s">
-        <v>1455</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33734,7 +33737,7 @@
         <v>295</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>1456</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33745,7 +33748,7 @@
         <v>294</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>1457</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33756,7 +33759,7 @@
         <v>293</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>1458</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33767,7 +33770,7 @@
         <v>296</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>1459</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33778,7 +33781,7 @@
         <v>292</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>1460</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33789,7 +33792,7 @@
         <v>291</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>1461</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33800,7 +33803,7 @@
         <v>290</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>1462</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33811,7 +33814,7 @@
         <v>289</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>1463</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33822,7 +33825,7 @@
         <v>288</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>1464</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33833,7 +33836,7 @@
         <v>261</v>
       </c>
       <c r="C45" s="30" t="s">
-        <v>1465</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33844,7 +33847,7 @@
         <v>260</v>
       </c>
       <c r="C46" s="30" t="s">
-        <v>1466</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33864,7 +33867,7 @@
         <v>258</v>
       </c>
       <c r="C48" s="30" t="s">
-        <v>1467</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33875,7 +33878,7 @@
         <v>257</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33886,7 +33889,7 @@
         <v>256</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>1469</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -33921,7 +33924,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C169"/>
-  <sheetFormatPr defaultColWidth="8.578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.578125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="22" width="8.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="22" width="3.43"/>
@@ -33931,1006 +33934,1006 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="22" t="s">
-        <v>1470</v>
+        <v>1471</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>1471</v>
+        <v>1472</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="s">
-        <v>1472</v>
+        <v>1473</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>1473</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="s">
-        <v>1474</v>
+        <v>1475</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>1475</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="s">
-        <v>1476</v>
+        <v>1477</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>1477</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="22" t="s">
-        <v>1478</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="22" t="s">
-        <v>1479</v>
+        <v>1480</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="22" t="s">
-        <v>1480</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="22" t="s">
-        <v>1481</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>1482</v>
+        <v>1483</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>1483</v>
+        <v>1484</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>1484</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>1485</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="s">
-        <v>1486</v>
+        <v>1487</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>1487</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="22" t="s">
-        <v>1488</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="22" t="s">
-        <v>1489</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="22" t="s">
-        <v>1490</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="22" t="s">
-        <v>1491</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="22" t="s">
-        <v>1492</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>1493</v>
+        <v>1494</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>1494</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="22" t="s">
-        <v>1495</v>
+        <v>1496</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>1496</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="22" t="s">
-        <v>1497</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="22" t="s">
-        <v>1498</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
-        <v>1499</v>
+        <v>1500</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>1500</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="22" t="s">
-        <v>1501</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="22" t="s">
-        <v>1502</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="22" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="22" t="s">
-        <v>1504</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="22" t="s">
-        <v>1505</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="22" t="s">
-        <v>1506</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="22" t="s">
-        <v>1507</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="22" t="s">
-        <v>1508</v>
+        <v>1509</v>
       </c>
       <c r="B30" s="22" t="s">
-        <v>1509</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="22" t="s">
-        <v>1510</v>
+        <v>1511</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="22" t="s">
-        <v>1511</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="22" t="s">
-        <v>1512</v>
+        <v>1513</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="22" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="22" t="s">
-        <v>1515</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="22" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="22" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="22" t="s">
-        <v>1518</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1519</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="55.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C39" s="32" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="22" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="B40" s="22" t="s">
-        <v>1521</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="22" t="s">
-        <v>1522</v>
+        <v>1523</v>
       </c>
       <c r="B41" s="22" t="s">
-        <v>1523</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="22" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="22" t="s">
-        <v>1525</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="22" t="s">
-        <v>1526</v>
+        <v>1527</v>
       </c>
       <c r="B44" s="22" t="s">
-        <v>1527</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="22" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="22" t="s">
-        <v>1529</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="22" t="s">
-        <v>1530</v>
+        <v>1531</v>
       </c>
       <c r="B47" s="22" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="22" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
       <c r="B48" s="22" t="s">
-        <v>1533</v>
+        <v>1534</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="22" t="s">
-        <v>1534</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="22" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
       <c r="B50" s="22" t="s">
-        <v>1536</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="22" t="s">
-        <v>1537</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="22" t="s">
-        <v>1538</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="22" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="22" t="s">
-        <v>1540</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="B55" s="22" t="s">
-        <v>1542</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="22" t="s">
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="B56" s="22" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="22" t="s">
-        <v>1545</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="22" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="22" t="s">
-        <v>1547</v>
+        <v>1548</v>
       </c>
       <c r="B59" s="22" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="22" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="22" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="B61" s="22" t="s">
-        <v>1551</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="22" t="s">
-        <v>1552</v>
+        <v>1553</v>
       </c>
       <c r="B62" s="22" t="s">
-        <v>1553</v>
+        <v>1554</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="22" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="B63" s="22" t="s">
-        <v>1555</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="22" t="s">
-        <v>1556</v>
+        <v>1557</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="22" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="22" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>1561</v>
+        <v>1562</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="22" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="B67" s="22" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="22" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
       <c r="B68" s="22" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="22" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
       <c r="B69" s="22" t="s">
-        <v>1567</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="22" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="22" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="22" t="s">
-        <v>1570</v>
+        <v>1571</v>
       </c>
       <c r="B72" s="22" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="22" t="s">
-        <v>1572</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="22" t="s">
-        <v>1573</v>
+        <v>1574</v>
       </c>
       <c r="B74" s="22" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="22" t="s">
-        <v>1575</v>
+        <v>1576</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="22" t="s">
-        <v>1576</v>
+        <v>1577</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="22" t="s">
-        <v>1577</v>
+        <v>1578</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="22" t="s">
-        <v>1578</v>
+        <v>1579</v>
       </c>
       <c r="B78" s="22" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="22" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="B79" s="22" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="22" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="B80" s="22" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="22" t="s">
-        <v>1584</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="22" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="B82" s="22" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="22" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="22" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="B84" s="22" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="22" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
       <c r="B85" s="22" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="22" t="s">
-        <v>1592</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="22" t="s">
-        <v>1593</v>
+        <v>1594</v>
       </c>
       <c r="B87" s="22" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="22" t="s">
-        <v>1595</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="22" t="s">
-        <v>1596</v>
+        <v>1597</v>
       </c>
       <c r="B89" s="22" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="22" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="22" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="B91" s="22" t="s">
-        <v>1600</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="22" t="s">
-        <v>1601</v>
+        <v>1602</v>
       </c>
       <c r="B92" s="22" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="22" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="22" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="22" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="22" t="s">
-        <v>1606</v>
+        <v>1607</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="22" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
       <c r="B97" s="22" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="22" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="22" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
       <c r="B99" s="22" t="s">
-        <v>1611</v>
+        <v>1612</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="22" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="22" t="s">
-        <v>1613</v>
+        <v>1614</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="22" t="s">
-        <v>1614</v>
+        <v>1615</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="22" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="22" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="B104" s="22" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="22" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="22" t="s">
-        <v>1619</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="22" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="22" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="22" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B110" s="22" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="22" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
       <c r="B111" s="22" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B112" s="22" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B113" s="22" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B114" s="22" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B115" s="22" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="22" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B117" s="22" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B118" s="22" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="22" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="B119" s="22" t="s">
-        <v>1634</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B120" s="22" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B121" s="22" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B122" s="22" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B123" s="22" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B124" s="22" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B125" s="22" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="22" t="s">
-        <v>1641</v>
+        <v>1642</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="22" t="s">
-        <v>1642</v>
+        <v>1643</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B128" s="22" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="22" t="s">
-        <v>1644</v>
+        <v>1645</v>
       </c>
       <c r="B129" s="22" t="s">
-        <v>1645</v>
+        <v>1646</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="22" t="s">
-        <v>1646</v>
+        <v>1647</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="22" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="22" t="s">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="22" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B134" s="22" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="22" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="B135" s="22" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B136" s="22" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B137" s="22" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B138" s="22" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="22" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="B139" s="22" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="22" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B141" s="22" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B142" s="22" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B143" s="22" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B144" s="22" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B145" s="22" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B146" s="22" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="22" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="B147" s="22" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B148" s="22" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B149" s="22" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="22" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="22" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="22" t="s">
-        <v>1671</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B153" s="22" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B154" s="22" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B155" s="22" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B156" s="22" t="s">
-        <v>1675</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B157" s="22" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="22" t="s">
-        <v>1677</v>
+        <v>1678</v>
       </c>
       <c r="B158" s="22" t="s">
-        <v>1678</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B159" s="22" t="s">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="22" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="22" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B162" s="22" t="s">
-        <v>1682</v>
+        <v>1683</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="22" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="B163" s="22" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B164" s="22" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B165" s="22" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="22" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B167" s="22" t="s">
-        <v>1687</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="22" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="22" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="B169" s="22" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
     </row>
   </sheetData>

</xml_diff>